<commit_message>
fix: fill all columns in RPM/wellness ICP report (wrist_reason, qual_status, revenue)
</commit_message>
<xml_diff>
--- a/marketing_vb/workspace/research/corporate-wellness-rpm/corporate_wellness_rpm_icp_scoring_report.xlsx
+++ b/marketing_vb/workspace/research/corporate-wellness-rpm/corporate_wellness_rpm_icp_scoring_report.xlsx
@@ -468,13 +468,13 @@
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
     <col width="55" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="55" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
     <col width="45" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
@@ -580,7 +580,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Insurance wellness / rewards</t>
+          <t>Insurance wellness rewards</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
@@ -600,10 +600,15 @@
           <t>Manulife Financial Corporation (NYSE/TSE: MFC) ($54.64B (Manulife, FY2024))</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>YES — Apple Watch is core to Vitality PLUS. Members earn Apple Watch through healthy behaviors. Wrist-worn device central to value proposition (10+ year program).</t>
+        </is>
+      </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>$54.64B (Manulife, FY2024)</t>
+          <t>$54.64B (Manulife, FY2024)
+https://stockanalysis.com/stocks/mfc/revenue/</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
@@ -621,8 +626,16 @@
           <t>John Hancock Announces Longer. Healthier. Better. Network — John Hancock, May 27, 2026 — https://www.johnhancock.com/about-us/news/john-hancock/2026/05/john-hancock-announces-longer-healthier-better-network-for-financial-professionals</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr"/>
-      <c r="P2" s="3" t="inlineStr"/>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=True</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -660,10 +673,15 @@
           <t>AIA Group Limited (HKEX: 1299) (~$20B+ (AIA Group total revenue FY2024))</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>YES — AIA Vitality links with fitness devices (Huawei, Garmin, Apple Watch, Samsung, Fitbit). Wrist devices integral to wellness engagement model.</t>
+        </is>
+      </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>~$20B+ (AIA Group total revenue FY2024)</t>
+          <t>~$20B+ (AIA Group total revenue FY2024)
+https://www.aia.com/content/dam/group-wise/en/docs/investor-relations/2025/AIA+Group+2024+Annual+Results+Ann+(Eng).pdf</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
@@ -681,8 +699,16 @@
           <t>Tata AIA introduces Indian consumers to Vitality — FM Live, 2025 — https://www.fmlive.in/tata-aia-introduces-indian-consumers-to-vitality-a-globally-renowned-holistic-wellness-program/</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr"/>
-      <c r="P3" s="3" t="inlineStr"/>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=True</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -700,7 +726,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Wearable DHT for clinical trials</t>
+          <t>Wearable DHT clinical trials</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
@@ -727,8 +753,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>~$150M (Signant Health est.)
-N/A</t>
+          <t>~$150M (Signant Health est.)</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -743,8 +768,7 @@
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>Signant Health Buys Ametris to Unite Data Streams in Clinical Trials — FierceBiotech, May 14, 2026
-https://www.fiercebiotech.com/cro/signant-health-buys-ametris-unite-data-streams-clinical-trials</t>
+          <t>Signant Health Buys Ametris to Unite Data Streams in Clinical Trials — FierceBiotech, May 14, 2026</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
@@ -774,7 +798,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>RPM + clinical trials (wrist)</t>
+          <t>RPM + trials (wrist)</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
@@ -791,13 +815,17 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Independent (life sciences division acquired by ActiGraph Jan 2025) (N/A)</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr"/>
+          <t>Independent (life sciences division acquired by ActiGraph Jan 2025)</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>YES — Biovitals platform uses FDA-cleared wearable sensors including wrist-worn devices for continuous RPM. FDA Breakthrough Device Designation for heart failure DTx. Wrist/wearable monitoring is core product.</t>
+        </is>
+      </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>https://getlatka.com/companies/biofourmis.com</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
@@ -815,8 +843,16 @@
           <t>ActiGraph Accelerates Clinical Trial Modernization with Transformational Acquisition of Biofourmis Life Science Business — PR Newswire, January 7, 2025 — https://www.prnewswire.com/news-releases/actigraph-accelerates-clinical-trial-modernization-with-transformational-acquisition-of-biofourmis-life-science-business-302344216.html</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr"/>
-      <c r="P5" s="3" t="inlineStr"/>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=True</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -834,7 +870,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Endpoint data + wearable sensors</t>
+          <t>Endpoint data + wearables</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
@@ -877,8 +913,7 @@
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>Thermo Fisher Completes $8.875 Billion Acquisition of Clario — Applied Clinical Trials, March 24, 2026
-https://www.appliedclinicaltrialsonline.com/view/thermo-fisher-acquisition-clario-clinical-trial-data</t>
+          <t>Thermo Fisher Completes $8.875 Billion Acquisition of Clario — Applied Clinical Trials, March 24, 2026</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
@@ -908,7 +943,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Insurer rewards ecosystem</t>
+          <t>Insurer rewards</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
@@ -928,10 +963,15 @@
           <t>Discovery Limited (JSE: DSY) (Group operating profit R11.6B (~$650M) FY2024; revenue ~$5B+)</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>YES — Core Vitality program integrates with fitness wearables (Apple Watch, Garmin, Samsung, Suunto, Fitbit). Points for step tracking, heart rate via wrist-worn devices.</t>
+        </is>
+      </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Group operating profit R11.6B (~$650M) FY2024; revenue ~$5B+</t>
+          <t>Group operating profit R11.6B (~$650M) FY2024; revenue ~$5B+
+https://www.discovery.co.za/assets/discoverycoza/corporate/investor-relations/2024/results-booklet-fy-2024.pdf</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
@@ -949,8 +989,16 @@
           <t>Discovery Vitality tricks the brain into healthier habits — MyBroadband / Daily Investor, 2025 — https://dailyinvestor.com/finance/59978/90000-coffees-and-r36-million-how-discovery-vitality-tricks-your-brain/</t>
         </is>
       </c>
-      <c r="O7" s="3" t="inlineStr"/>
-      <c r="P7" s="3" t="inlineStr"/>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=True</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -968,7 +1016,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Unified trial solution + RPM</t>
+          <t>Unified trial + RPM</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
@@ -988,10 +1036,15 @@
           <t>AstraZeneca (launched as separate health-tech business, Nov 2023) ($54.1B (AstraZeneca, FY2024))</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Unified trial solution supports digital wearables, sensors, and connected medical devices for data collection. Integrates wearables but does not deploy proprietary wrist devices as sole offering.</t>
+        </is>
+      </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>$54.1B (AstraZeneca, FY2024)</t>
+          <t>$54.1B (AstraZeneca, FY2024)
+https://prospeo.io/c/evinova-revenue</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
@@ -1009,8 +1062,16 @@
           <t>Evinova Announces Strategic Collaborations with Astellas, AstraZeneca and Bristol Myers Squibb — Evinova Press Release, February 18, 2026 — https://evinova.com/press-releases</t>
         </is>
       </c>
-      <c r="O8" s="3" t="inlineStr"/>
-      <c r="P8" s="3" t="inlineStr"/>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>Seed-list exception</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=False</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1045,7 +1106,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>None (public: NASDAQ MASI) (N/A)</t>
+          <t>None (public: NASDAQ MASI)</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -1055,8 +1116,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>N/A
-https://stockanalysis.com/stocks/masi/revenue/</t>
+          <t>https://stockanalysis.com/stocks/masi/revenue/</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
@@ -1071,8 +1131,7 @@
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>Masimo Reports Fourth Quarter and Full-Year 2024 Financial Results — BusinessWire, February 25, 2025
-https://www.businesswire.com/news/home/20250225391908/en/Masimo-Reports-Fourth-Quarter-and-Full-Year-2024-Financial-Results</t>
+          <t>Masimo Reports Fourth Quarter and Full-Year 2024 Financial Results — BusinessWire, February 25, 2025</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
@@ -1145,8 +1204,7 @@
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>Signant Health Buys Ametris to Unite Data Streams in Clinical Trials — FierceBiotech, May 14, 2026
-https://www.fiercebiotech.com/cro/signant-health-buys-ametris-unite-data-streams-clinical-trials</t>
+          <t>Signant Health Buys Ametris to Unite Data Streams in Clinical Trials — FierceBiotech, May 14, 2026</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr">
@@ -1176,7 +1234,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Employer wellbeing platform</t>
+          <t>Employer wellbeing</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
@@ -1196,10 +1254,15 @@
           <t>Discovery Limited (JSE: DSY) (~$5B+ (Discovery Limited group revenue FY2024))</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>YES — Vitality program integrates with fitness wearables (Apple Watch, Garmin, Samsung, Fitbit). Wrist devices central to behavior-change, points-based wellness model.</t>
+        </is>
+      </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>~$5B+ (Discovery Limited group revenue FY2024)</t>
+          <t>~$5B+ (Discovery Limited group revenue FY2024)
+https://rocketreach.co/vitality-group-inc-profile_b5c039c1f42e0822</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
@@ -1217,8 +1280,16 @@
           <t>Vitality and Google Partner to Bring AI-Powered Health Solutions to Millions — PR Newswire, November 4, 2025 — https://www.prnewswire.com/news-releases/vitality-and-google-partner-to-bring-ai-powered-health-solutions-to-millions-302604260.html</t>
         </is>
       </c>
-      <c r="O11" s="3" t="inlineStr"/>
-      <c r="P11" s="3" t="inlineStr"/>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=True</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1236,7 +1307,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Insurtech / wellbeing app</t>
+          <t>Insurtech wellbeing</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
@@ -1253,13 +1324,17 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Independent (private, unicorn)</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr"/>
+          <t>Independent (private, unicorn) ($72M ARR (2024))</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Betterfly is an insurtech/corporate wellness benefits platform that rewards employees' healthy habits with insurance benefits and charitable donations. No evidence of deploying wrist-worn devices. Platform integrates with fitness apps but does not provide hardware.</t>
+        </is>
+      </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t>$72M ARR (2024)
 https://getlatka.com/companies/betterfly.com</t>
         </is>
       </c>
@@ -1283,7 +1358,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P12" s="3" t="inlineStr"/>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>funding: $202.5M raised (Series C, $1B valuation unicorn)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1318,7 +1397,7 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>None (independent) (N/A)</t>
+          <t>None (independent)</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
@@ -1328,8 +1407,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>N/A
-https://www.cbinsights.com/company/biobeat/financials</t>
+          <t>https://www.cbinsights.com/company/biobeat/financials</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
@@ -1344,8 +1422,7 @@
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>Biobeat Secures $50 Million Series B Financing to Advance Cuffless Blood Pressure Monitoring — Yahoo Finance, December 31, 2025
-https://finance.yahoo.com/news/biobeat-secures-50-million-series-213900421.html</t>
+          <t>Biobeat Secures $50 Million Series B Financing to Advance Cuffless Blood Pressure Monitoring — Yahoo Finance, December 31, 2025</t>
         </is>
       </c>
       <c r="O13" s="3" t="inlineStr">
@@ -1375,7 +1452,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Virtual wards + monitoring</t>
+          <t>Virtual wards</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
@@ -1395,8 +1472,16 @@
           <t>Independent (private, Series B)</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr"/>
-      <c r="K14" s="3" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Doccla has launched a wrist-worn device for passive vital sign monitoring that streams data to their clinical dashboard. Used specifically for monitoring acutely unwell patients (e.g., Cytokine Release Syndrome). Confirmed via LinkedIn post from Doccla's team and TechCrunch coverage showing 'finger to wrist-worn monitor' imagery.</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
           <t>https://www.doccla.com</t>
@@ -1417,7 +1502,11 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="P14" s="3" t="inlineStr"/>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>funding: $72.5M raised (Series B: $46M, Sep 2024)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1435,7 +1524,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Payer wellness + rewards</t>
+          <t>Payer wellness rewards</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
@@ -1455,10 +1544,15 @@
           <t>Humana Inc. (NYSE: HUM) ($106.37B (Humana, FY2024))</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>YES — Go365 integrates with fitness trackers/smartwatches (Fitbit, Garmin, Apple Watch, Samsung). Wrist-worn devices are essential for activity tracking and rewards.</t>
+        </is>
+      </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>$106.37B (Humana, FY2024)</t>
+          <t>$106.37B (Humana, FY2024)
+https://wellness.go365.com/about-us</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
@@ -1476,8 +1570,16 @@
           <t>Humana Go365 Wellness and Rewards Program Announces Five-Year Impact Study Results — MarketScreener, 2025 — https://www.marketscreener.com/quote/stock/HUMANA-INC-13000/news/Humana-Go365-Wellness-and-Rewards-Program-Announces-Five-Year-Impact-Study-Results-29020729/</t>
         </is>
       </c>
-      <c r="O15" s="3" t="inlineStr"/>
-      <c r="P15" s="3" t="inlineStr"/>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=True</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1515,10 +1617,15 @@
           <t>Public (NASDAQ: ICLR) ($8.28B (ICON, FY2024))</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Major global CRO. Early investment in mobile health through PRA acquisition. Supports wearables in trials but no proprietary wrist device as core product.</t>
+        </is>
+      </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>$8.28B (ICON, FY2024)</t>
+          <t>$8.28B (ICON, FY2024)
+https://investor.iconplc.com/news-releases/news-release-details/icon-reports-fourth-quarter-and-full-year-2024-results</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
@@ -1536,8 +1643,16 @@
           <t>The Clinical Crisis: A Deep-Dive Into ICON plc Amidst a Transformational Storm — FinancialContent, February 12, 2026 — https://markets.financialcontent.com/wral/article/finterra-2026-2-12-the-clinical-crisis-a-deep-dive-into-icon-plc-iclr-amidst-a-transformational-storm</t>
         </is>
       </c>
-      <c r="O16" s="3" t="inlineStr"/>
-      <c r="P16" s="3" t="inlineStr"/>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>Seed-list exception</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=False</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1555,7 +1670,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Large CRO / trial-tech</t>
+          <t>CRO / trial-tech</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
@@ -1575,10 +1690,15 @@
           <t>Public (NYSE: IQV) ($15.4B (IQVIA, FY2024))</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr"/>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Large CRO with RPM and digital health capabilities. AI-driven RPM white paper covers wearable devices. Integrates third-party devices but no proprietary wrist device as core product.</t>
+        </is>
+      </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>$15.4B (IQVIA, FY2024)</t>
+          <t>$15.4B (IQVIA, FY2024)
+https://www.iqvia.com/newsroom/2025/02/iqvia-reports-fourth-quarter-and-full-year-2024-results</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
@@ -1596,8 +1716,16 @@
           <t>Innovating the Digital Care Model — IQVIA Blog, March 6, 2026 — https://www.iqvia.com/blogs/2026/03/innovating-the-digital-care-model</t>
         </is>
       </c>
-      <c r="O17" s="3" t="inlineStr"/>
-      <c r="P17" s="3" t="inlineStr"/>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>Seed-list exception</t>
+        </is>
+      </c>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=False</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1615,7 +1743,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Decentralized trials platform</t>
+          <t>Decentralized trials</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
@@ -1632,7 +1760,7 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>None (independent) (N/A)</t>
+          <t>None (independent)</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
@@ -1642,8 +1770,7 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>N/A
-https://getlatka.com/companies/medable-1</t>
+          <t>https://getlatka.com/companies/medable-1</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
@@ -1658,8 +1785,7 @@
       </c>
       <c r="N18" s="3" t="inlineStr">
         <is>
-          <t>Medable Launches The Industry's First Agentic AI Platform and CRA Agent — BusinessWire, September 3, 2025
-https://www.businesswire.com/news/home/20250903949263/en/Medable-Launches-The-Industrys-First-Agentic-AI-Platform-and-CRA-Agent-Removes-Bottlenecks-in-Clinical-Development</t>
+          <t>Medable Launches The Industry's First Agentic AI Platform and CRA Agent — BusinessWire, September 3, 2025</t>
         </is>
       </c>
       <c r="O18" s="3" t="inlineStr">
@@ -1689,7 +1815,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Sensor platform for trials</t>
+          <t>Sensor platform trials</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
@@ -1732,8 +1858,7 @@
       </c>
       <c r="N19" s="3" t="inlineStr">
         <is>
-          <t>Medidata Launches Clinical Data Studio, Leveraging AI to Modernize Data Experience in Clinical Trials — Dassault Systèmes Press Release, June 18, 2024
-https://www.3ds.com/newsroom/press-releases/medidata-launches-clinical-data-studio-leveraging-ai-modernize-data-experience-clinical-trials</t>
+          <t>Medidata Launches Clinical Data Studio, Leveraging AI to Modernize Data Experience in Clinical Trials — Dassault Systèmes Press Release, June 18, 2024</t>
         </is>
       </c>
       <c r="O19" s="3" t="inlineStr">
@@ -1763,7 +1888,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>CRO — DCT wearables</t>
+          <t>CRO DCT wearables</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
@@ -1783,10 +1908,15 @@
           <t>EQT Private Equity / Goldman Sachs Asset Management ($3.78B (Parexel, FY2024 est.))</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr"/>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Top-10 global CRO. Full-service clinical development. No proprietary wrist device; platform-agnostic approach to wearables in trials.</t>
+        </is>
+      </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>$3.78B (Parexel, FY2024 est.)</t>
+          <t>$3.78B (Parexel, FY2024 est.)
+https://rocketreach.co/parexel-profile_b5c608b1f42e0c53</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
@@ -1804,8 +1934,16 @@
           <t>Parexel Launches ParexelAI Suite of Human-Led AI Services for Clinical Development — HIT Consultant, May 18, 2026 — https://hitconsultant.net/2026/05/18/parexel-launches-parexelai-clinical-development-suite/</t>
         </is>
       </c>
-      <c r="O20" s="3" t="inlineStr"/>
-      <c r="P20" s="3" t="inlineStr"/>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>Seed-list exception</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=False</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1823,7 +1961,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Employer wellbeing / rewards</t>
+          <t>Employer wellbeing/rewards</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
@@ -1843,10 +1981,15 @@
           <t>New Mountain Capital (Virgin Pulse + HealthComp merged, Nov 2023) ($500M+ (Personify Health, FY2024))</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr"/>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>YES — Deploys Max GO wrist-worn activity tracking device that syncs to the Personify Health platform. Wrist wearables are a key engagement tool for corporate wellness programs.</t>
+        </is>
+      </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>$500M+ (Personify Health, FY2024)</t>
+          <t>$500M+ (Personify Health, FY2024)
+https://endpoints.news/personify-health-shares-2024-revenue-profitability/</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr">
@@ -1864,8 +2007,16 @@
           <t>McCabe named CEO of Personify Health — Providence Business News, January 14, 2025 — https://pbn.com/mccabe-named-ceo-of-personify-health/</t>
         </is>
       </c>
-      <c r="O21" s="3" t="inlineStr"/>
-      <c r="P21" s="3" t="inlineStr"/>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="P21" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=True</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1883,7 +2034,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Direct-to-patient trial site</t>
+          <t>Direct-to-patient trials</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
@@ -1926,8 +2077,7 @@
       </c>
       <c r="N22" s="3" t="inlineStr">
         <is>
-          <t>Science 37 Agrees to Be Acquired by eMed in Deal Valued at $38M — FierceBiotech, January 29, 2024
-https://www.fiercebiotech.com/cro/science-37-agrees-be-acquired-emed-deal-valued-38m</t>
+          <t>Science 37 Agrees to Be Acquired by eMed in Deal Valued at $38M — FierceBiotech, January 29, 2024</t>
         </is>
       </c>
       <c r="O22" s="3" t="inlineStr">
@@ -1957,7 +2107,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Decentralized / hybrid trials</t>
+          <t>Decentralized/hybrid trials</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
@@ -1974,13 +2124,17 @@
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Independent (N/A)</t>
-        </is>
-      </c>
-      <c r="J23" s="3" t="inlineStr"/>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Cloud-based EDC/ePRO/eCOA platform. Integrates with wearables and medical devices but does not deploy proprietary wrist devices as core product.</t>
+        </is>
+      </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>https://growjo.com/company/Castor_EDC</t>
         </is>
       </c>
       <c r="L23" s="3" t="inlineStr">
@@ -1998,8 +2152,16 @@
           <t>Castor Accelerating Global Medical Device Research With Decentralized Clinical Trials Platform — BioSpace, 2025 — https://www.biospace.com/castor-accelerating-global-medical-device-research-with-decentralized-clinical-trials-platform</t>
         </is>
       </c>
-      <c r="O23" s="3" t="inlineStr"/>
-      <c r="P23" s="3" t="inlineStr"/>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t>Seed-list exception</t>
+        </is>
+      </c>
+      <c r="P23" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=False</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -2034,7 +2196,7 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>None (MIT Media Lab spin-off) (N/A)</t>
+          <t>None (MIT Media Lab spin-off)</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
@@ -2044,8 +2206,7 @@
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>N/A
-https://www.signalhire.com/companies/empatica</t>
+          <t>https://www.signalhire.com/companies/empatica</t>
         </is>
       </c>
       <c r="L24" s="3" t="inlineStr">
@@ -2060,8 +2221,7 @@
       </c>
       <c r="N24" s="3" t="inlineStr">
         <is>
-          <t>Empatica's Platform Receives New FDA Clearance for Cardiac Digital Biomarkers — ClinLab International, 2025
-https://clinlabint.com/empaticas-platform-receives-new-fda-clearance-for-cardiac-digital-biomarkers/</t>
+          <t>Empatica's Platform Receives New FDA Clearance for Cardiac Digital Biomarkers — ClinLab International, 2025</t>
         </is>
       </c>
       <c r="O24" s="3" t="inlineStr">
@@ -2091,7 +2251,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Digital biomarker / wearable platform</t>
+          <t>Digital biomarker wearable</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
@@ -2108,7 +2268,7 @@
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>None (independent) (N/A)</t>
+          <t>None (independent)</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
@@ -2118,8 +2278,7 @@
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>N/A
-https://compworth.com/company/koneksa-health</t>
+          <t>https://compworth.com/company/koneksa-health</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr">
@@ -2134,8 +2293,7 @@
       </c>
       <c r="N25" s="3" t="inlineStr">
         <is>
-          <t>Koneksa to Study if AI Smartwatch Data Can Predict Parkinson's Progression Using Verily's Clinical Smartwatch — FierceBiotech, 2025
-https://www.fiercebiotech.com/medtech/koneksa-study-whether-ai-analyzed-smartwatch-data-can-predict-parkinsons-progression</t>
+          <t>Koneksa to Study if AI Smartwatch Data Can Predict Parkinson's Progression Using Verily's Clinical Smartwatch — FierceBiotech, 2025</t>
         </is>
       </c>
       <c r="O25" s="3" t="inlineStr">
@@ -2165,7 +2323,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Remote monitoring platform</t>
+          <t>Remote monitoring</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
@@ -2182,13 +2340,17 @@
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>OMRON Healthcare</t>
-        </is>
-      </c>
-      <c r="J26" s="3" t="inlineStr"/>
+          <t>OMRON Healthcare ($7.7M ARR (2025))</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>Luscii provides a remote patient monitoring platform used in ~70% of Dutch hospitals. Parent company OMRON manufactures wrist BP monitors, but Luscii's platform integrates various devices without specifically deploying wrist-worn devices as a core offering.</t>
+        </is>
+      </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t>$7.7M ARR (2025)
 https://getlatka.com/companies/luscii.com</t>
         </is>
       </c>
@@ -2212,7 +2374,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P26" s="3" t="inlineStr"/>
+      <c r="P26" s="3" t="inlineStr">
+        <is>
+          <t>funding: Acquired by OMRON Healthcare (undisclosed)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -2273,8 +2439,7 @@
       </c>
       <c r="N27" s="3" t="inlineStr">
         <is>
-          <t>The Buyback Pays Off: Withings Confirms Full-Year Profitability for 2025 Driven by US Market Dominance — PRNewswire, June 30, 2026
-https://www.prnewswire.com/news-releases/the-buyback-pays-off-withings-confirms-full-year-profitability-for-2025-driven-by-us-market-dominance-302813605.html</t>
+          <t>The Buyback Pays Off: Withings Confirms Full-Year Profitability for 2025 Driven by US Market Dominance — PRNewswire, June 30, 2026</t>
         </is>
       </c>
       <c r="O27" s="3" t="inlineStr">
@@ -2321,13 +2486,17 @@
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>Independent (N/A)</t>
-        </is>
-      </c>
-      <c r="J28" s="3" t="inlineStr"/>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>DHEP platform integrates with wearables (fitness trackers, smartwatches, BP monitors, glucose monitors). Wrist devices feed Health Score but are not proprietary.</t>
+        </is>
+      </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>https://growjo.com/company/dacadoo</t>
         </is>
       </c>
       <c r="L28" s="3" t="inlineStr">
@@ -2345,8 +2514,16 @@
           <t>dacadoo Launches Gen 5 of Award-Winning Health Platform — HLTH, May 27, 2025 — https://hlth.com/insights/news/dacadoo-launches-gen-5-of-award-winning-health-platform-2025-05-27</t>
         </is>
       </c>
-      <c r="O28" s="3" t="inlineStr"/>
-      <c r="P28" s="3" t="inlineStr"/>
+      <c r="O28" s="3" t="inlineStr">
+        <is>
+          <t>Seed-list exception</t>
+        </is>
+      </c>
+      <c r="P28" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=False</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -2364,7 +2541,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Group insurance + wellbeing</t>
+          <t>Group insurance wellbeing</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
@@ -2381,13 +2558,17 @@
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>Independent (strategic investment from Dai-ichi Life) (N/A)</t>
-        </is>
-      </c>
-      <c r="J29" s="3" t="inlineStr"/>
+          <t>Independent (strategic investment from Dai-ichi Life)</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>App-based wellness and insurance platform with gamification. Integrates fitness tracking via smartphone and third-party wearables. No proprietary wrist device.</t>
+        </is>
+      </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>https://compworth.com/company/yulife</t>
         </is>
       </c>
       <c r="L29" s="3" t="inlineStr">
@@ -2405,8 +2586,16 @@
           <t>Sodexo and YuLife Recognise World Wellbeing Week — Insurance Edge, June 27, 2025 — https://insurance-edge.net/2025/06/27/sodexo-and-yulife-recognise-world-wellbeing-week/</t>
         </is>
       </c>
-      <c r="O29" s="3" t="inlineStr"/>
-      <c r="P29" s="3" t="inlineStr"/>
+      <c r="O29" s="3" t="inlineStr">
+        <is>
+          <t>Seed-list exception</t>
+        </is>
+      </c>
+      <c r="P29" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=False</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -2424,7 +2613,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>eCOA platform + wearables</t>
+          <t>eCOA + wearables</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
@@ -2444,10 +2633,15 @@
           <t>Eli Lilly and Company (acquired July 2024) ($45B (Eli Lilly, FY2024))</t>
         </is>
       </c>
-      <c r="J30" s="3" t="inlineStr"/>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>YES — Atom5 platform uses wearable wristbands (Garmin partnership) for continuous patient monitoring in clinical trials. Wrist-worn wearables are core to the data capture methodology.</t>
+        </is>
+      </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>$45B (Eli Lilly, FY2024)</t>
+          <t>$45B (Eli Lilly, FY2024)
+https://www.crunchbase.com/organization/aparito</t>
         </is>
       </c>
       <c r="L30" s="3" t="inlineStr">
@@ -2465,8 +2659,16 @@
           <t>Welsh medtech venture Aparito acquired by US firm Eli Lilly — Business Live, July 11, 2024 — https://www.business-live.co.uk/technology/welsh-medtech-venture-aparito-acquired-29524813</t>
         </is>
       </c>
-      <c r="O30" s="3" t="inlineStr"/>
-      <c r="P30" s="3" t="inlineStr"/>
+      <c r="O30" s="3" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="P30" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=True</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -2501,7 +2703,7 @@
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>None (independent) (N/A)</t>
+          <t>None (independent)</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
@@ -2511,8 +2713,7 @@
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>N/A
-https://prospeo.io/c/biostrap-revenue</t>
+          <t>https://prospeo.io/c/biostrap-revenue</t>
         </is>
       </c>
       <c r="L31" s="3" t="inlineStr">
@@ -2527,8 +2728,7 @@
       </c>
       <c r="N31" s="3" t="inlineStr">
         <is>
-          <t>Biostrap Launches Kairos Wrist-Worn Digital Health Monitoring Device for Stress Resilience — MassDevice, 2023
-https://www.massdevice.com/biostrap-launches-wearable-health-monitoring-device/</t>
+          <t>Biostrap Launches Kairos Wrist-Worn Digital Health Monitoring Device for Stress Resilience — MassDevice, 2023</t>
         </is>
       </c>
       <c r="O31" s="3" t="inlineStr">
@@ -2575,7 +2775,7 @@
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>None (independent) (N/A)</t>
+          <t>None (independent)</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
@@ -2585,8 +2785,7 @@
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>N/A
-N/A</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="L32" s="3" t="inlineStr">
@@ -2601,8 +2800,7 @@
       </c>
       <c r="N32" s="3" t="inlineStr">
         <is>
-          <t>CardiacSense Valuation Drops Nearly 85% in One Year — TechTime News, July 4, 2025
-https://techtime.news/2025/07/04/cardiacsense/</t>
+          <t>CardiacSense Valuation Drops Nearly 85% in One Year — TechTime News, July 4, 2025</t>
         </is>
       </c>
       <c r="O32" s="3" t="inlineStr">
@@ -2649,7 +2847,7 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND (N/A)</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
@@ -2659,8 +2857,7 @@
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>N/A
-N/A</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="L33" s="3" t="inlineStr">
@@ -2675,8 +2872,7 @@
       </c>
       <c r="N33" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND (limited public presence)
-N/A</t>
+          <t>NOT FOUND (limited public presence)</t>
         </is>
       </c>
       <c r="O33" s="3" t="inlineStr">
@@ -2706,7 +2902,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>RPM / RTM platform</t>
+          <t>RPM/RTM platform</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
@@ -2723,13 +2919,17 @@
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>Independent (private, Series C)</t>
-        </is>
-      </c>
-      <c r="J34" s="3" t="inlineStr"/>
+          <t>Independent (private, Series C) ($7.9M ARR (2025 est.))</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>Devices include cellular BP cuffs, smart scales, pulse oximeters, glucose meters, spirometers. No wrist-worn device identified.</t>
+        </is>
+      </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t>$7.9M ARR (2025 est.)
 https://getlatka.com/companies/coachcare.com</t>
         </is>
       </c>
@@ -2753,7 +2953,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P34" s="3" t="inlineStr"/>
+      <c r="P34" s="3" t="inlineStr">
+        <is>
+          <t>funding: $60.2M raised</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -2788,7 +2992,7 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>None (independent) (N/A)</t>
+          <t>None (independent)</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
@@ -2798,8 +3002,7 @@
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>N/A
-N/A</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr">
@@ -2814,8 +3017,7 @@
       </c>
       <c r="N35" s="3" t="inlineStr">
         <is>
-          <t>Medtronic Expands Acute Care &amp; Monitoring Portfolio in Europe with Distribution Agreement for Corsano Multi-Parameter Wearable — Med-Tech Insights, May 22, 2025
-https://med-techinsights.com/2025/05/22/medtronic-signs-agreement-with-corsano-to-distribute-wearables/</t>
+          <t>Medtronic Expands Acute Care &amp; Monitoring Portfolio in Europe with Distribution Agreement for Corsano Multi-Parameter Wearable — Med-Tech Insights, May 22, 2025</t>
         </is>
       </c>
       <c r="O35" s="3" t="inlineStr">
@@ -2845,7 +3047,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Remote / hybrid trial platform</t>
+          <t>Remote trial platform</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
@@ -2862,13 +3064,17 @@
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>Independent (N/A)</t>
-        </is>
-      </c>
-      <c r="J36" s="3" t="inlineStr"/>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>eClinical platform (ePRO, eConsent, EDC). Does not deploy proprietary wrist devices; platform-agnostic device integrations for DCTs.</t>
+        </is>
+      </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>https://getlatka.com/companies/curebase.com</t>
         </is>
       </c>
       <c r="L36" s="3" t="inlineStr">
@@ -2886,8 +3092,16 @@
           <t>Curebase Expands AI-Powered eClinical Platform and Launches Sitebase — Clinical Research News Online, January 30, 2026 — https://www.clinicalresearchnewsonline.com/news/2026/01/30/curebase-expands-ai-powered-eclinical-platform-and-launches-sitebase-free-modern-technology-for-research-sites</t>
         </is>
       </c>
-      <c r="O36" s="3" t="inlineStr"/>
-      <c r="P36" s="3" t="inlineStr"/>
+      <c r="O36" s="3" t="inlineStr">
+        <is>
+          <t>Seed-list exception</t>
+        </is>
+      </c>
+      <c r="P36" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=False</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -2925,8 +3139,16 @@
           <t>Independent (private)</t>
         </is>
       </c>
-      <c r="J37" s="3" t="inlineStr"/>
-      <c r="K37" s="3" t="inlineStr"/>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>HRS provides disease-specific care plans with connected devices including BP monitors, weight scales, pulse oximeters, and glucose meters. No wrist-worn device deployment identified.</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
           <t>https://www.healthrecoverysolutions.com</t>
@@ -2947,7 +3169,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P37" s="3" t="inlineStr"/>
+      <c r="P37" s="3" t="inlineStr">
+        <is>
+          <t>funding: NOT FOUND</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -2982,13 +3208,17 @@
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>Independent (strategic investment from Guardant Health) (N/A)</t>
-        </is>
-      </c>
-      <c r="J38" s="3" t="inlineStr"/>
+          <t>Independent (strategic investment from Guardant Health)</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>Decentralized clinical trial platform (ObvioGo). Partners with device manufacturers for trials; does not deploy proprietary wrist-worn RPM devices as core product.</t>
+        </is>
+      </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>https://getlatka.com/companies/obviohealth</t>
         </is>
       </c>
       <c r="L38" s="3" t="inlineStr">
@@ -3006,8 +3236,16 @@
           <t>ObvioHealth Introduces ObvioGo 2.2: Transforming Study Management with AI-Driven Innovation — PR Newswire, January 14, 2025 — https://www.prnewswire.com/news/obviohealth/</t>
         </is>
       </c>
-      <c r="O38" s="3" t="inlineStr"/>
-      <c r="P38" s="3" t="inlineStr"/>
+      <c r="O38" s="3" t="inlineStr">
+        <is>
+          <t>Seed-list exception</t>
+        </is>
+      </c>
+      <c r="P38" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=False</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -3025,7 +3263,7 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>DHT-enabled decentralized trials</t>
+          <t>DHT decentralized trials</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
@@ -3042,13 +3280,17 @@
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>JLL Partners / Water Street (private equity backed) (NOT FOUND)</t>
-        </is>
-      </c>
-      <c r="J39" s="3" t="inlineStr"/>
+          <t>JLL Partners / Water Street (private equity backed)</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>Platform supports pre-built integrations with wearables and medical devices but no proprietary wrist device. Integrates third-party wearables for DCT/eCOA data capture.</t>
+        </is>
+      </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>https://tracxn.com/d/companies/thread/__Bq3zZ6N4vfHJKXH3ZACKkn_aBxOv4GW3Y6N87XFAwWs</t>
         </is>
       </c>
       <c r="L39" s="3" t="inlineStr">
@@ -3066,8 +3308,16 @@
           <t>THREAD Press Releases (latest March 2026) — THREAD, March 2026 — https://www.threadresearch.com/press-releases</t>
         </is>
       </c>
-      <c r="O39" s="3" t="inlineStr"/>
-      <c r="P39" s="3" t="inlineStr"/>
+      <c r="O39" s="3" t="inlineStr">
+        <is>
+          <t>Seed-list exception</t>
+        </is>
+      </c>
+      <c r="P39" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=False</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -3102,7 +3352,7 @@
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>None (independent) (N/A)</t>
+          <t>None (independent)</t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
@@ -3112,8 +3362,7 @@
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>N/A
-https://www.konaequity.com/company/validic-inc-4019063112/</t>
+          <t>https://www.konaequity.com/company/validic-inc-4019063112/</t>
         </is>
       </c>
       <c r="L40" s="3" t="inlineStr">
@@ -3128,8 +3377,7 @@
       </c>
       <c r="N40" s="3" t="inlineStr">
         <is>
-          <t>Validic Powers Scalable AI-Driven Remote Care at CES 2026 — Yahoo Finance, January 2026
-https://finance.yahoo.com/news/validic-powers-scalable-ai-driven-123000828.html</t>
+          <t>Validic Powers Scalable AI-Driven Remote Care at CES 2026 — Yahoo Finance, January 2026</t>
         </is>
       </c>
       <c r="O40" s="3" t="inlineStr">
@@ -3159,7 +3407,7 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Remote care + shipped devices</t>
+          <t>Remote care+devices</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
@@ -3176,13 +3424,17 @@
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Connect America</t>
-        </is>
-      </c>
-      <c r="J41" s="3" t="inlineStr"/>
+          <t>Connect America ($3.3M ARR (2025 est.))</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>100Plus provides RPM platform with BP monitors, glucose meters, pulse oximeters, and scales. No wrist-worn device identified. AI virtual assistant 'Ava' for care coordination.</t>
+        </is>
+      </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t>$3.3M ARR (2025 est.)
 https://getlatka.com/companies/100plus.com</t>
         </is>
       </c>
@@ -3206,7 +3458,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P41" s="3" t="inlineStr"/>
+      <c r="P41" s="3" t="inlineStr">
+        <is>
+          <t>funding: Acquired by Connect America (2021)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -3244,8 +3500,16 @@
           <t>Independent (private, founded 2002)</t>
         </is>
       </c>
-      <c r="J42" s="3" t="inlineStr"/>
-      <c r="K42" s="3" t="inlineStr"/>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>AMC Health provides end-to-end virtual care with real-time physiometric data, predictive AI, and clinical intervention. Device suite includes BP monitors, scales, pulse oximeters, glucose meters. No wrist-worn device identified.</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
       <c r="L42" s="3" t="inlineStr">
         <is>
           <t>https://www.amchealth.com</t>
@@ -3266,7 +3530,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P42" s="3" t="inlineStr"/>
+      <c r="P42" s="3" t="inlineStr">
+        <is>
+          <t>funding: NOT FOUND</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -3301,13 +3569,17 @@
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>Independent (private)</t>
-        </is>
-      </c>
-      <c r="J43" s="3" t="inlineStr"/>
+          <t>Independent (private) ($11.8M (estimated))</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>HUSK offers all-in-one corporate wellness benefits with challenges, rewards, telehealth nutrition, and mental health support. No evidence of deploying wrist-worn devices.</t>
+        </is>
+      </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t>$11.8M (estimated)
 https://compworth.com/company/huskwellnesscom</t>
         </is>
       </c>
@@ -3331,7 +3603,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P43" s="3" t="inlineStr"/>
+      <c r="P43" s="3" t="inlineStr">
+        <is>
+          <t>funding: NOT FOUND</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -3349,7 +3625,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Employee wellbeing platform</t>
+          <t>Employee wellbeing</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
@@ -3366,13 +3642,17 @@
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>H2 Wellbeing (independent)</t>
-        </is>
-      </c>
-      <c r="J44" s="3" t="inlineStr"/>
+          <t>H2 Wellbeing (independent) ($649.5K ARR (2024))</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>HeiaHeia partners with Polar for wearable integration (Polar x HeiaHeia corporate wellness). The platform syncs with wearables but does not deploy or provide its own wrist-worn devices.</t>
+        </is>
+      </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t>$649.5K ARR (2024)
 https://getlatka.com/companies/heiaheiacom</t>
         </is>
       </c>
@@ -3396,7 +3676,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P44" s="3" t="inlineStr"/>
+      <c r="P44" s="3" t="inlineStr">
+        <is>
+          <t>funding: ~$2M raised (2014 round + Tekes)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -3431,7 +3715,7 @@
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>None (independent) (N/A)</t>
+          <t>None (independent)</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
@@ -3441,8 +3725,7 @@
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>N/A
-N/A</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="L45" s="3" t="inlineStr">
@@ -3457,8 +3740,7 @@
       </c>
       <c r="N45" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND (minimal media presence)
-N/A</t>
+          <t>NOT FOUND (minimal media presence)</t>
         </is>
       </c>
       <c r="O45" s="3" t="inlineStr">
@@ -3488,7 +3770,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Remote care + cellular devices</t>
+          <t>Remote care+cellular</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
@@ -3505,13 +3787,17 @@
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>Independent (private)</t>
-        </is>
-      </c>
-      <c r="J46" s="3" t="inlineStr"/>
+          <t>Independent (private) ($12.1M ARR (2024 est.))</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>Prevounce provides cellular-connected patient devices for RPM including BP monitors, pulse oximeters, glucose meters, and scales. No wrist-worn device identified.</t>
+        </is>
+      </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t>$12.1M ARR (2024 est.)
 https://getlatka.com/companies/prevounce-health</t>
         </is>
       </c>
@@ -3535,7 +3821,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P46" s="3" t="inlineStr"/>
+      <c r="P46" s="3" t="inlineStr">
+        <is>
+          <t>funding: $4.5M–$7M raised</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -3553,7 +3843,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Cellular RPM device network</t>
+          <t>Cellular RPM network</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
@@ -3570,11 +3860,19 @@
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>Independent (private)</t>
-        </is>
-      </c>
-      <c r="J47" s="3" t="inlineStr"/>
-      <c r="K47" s="3" t="inlineStr"/>
+          <t>Independent (private) (NOT FOUND (recurring revenue 6x growth over 36 months))</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>Smart Meter provides cellular-connected RPM devices including BP monitors, glucose meters, pulse oximeters, weight scales, and thermometers. No wrist-worn device identified. 180K+ providers served.</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>NOT FOUND (recurring revenue 6x growth over 36 months)</t>
+        </is>
+      </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
           <t>https://smartmeterrpm.com</t>
@@ -3595,7 +3893,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P47" s="3" t="inlineStr"/>
+      <c r="P47" s="3" t="inlineStr">
+        <is>
+          <t>funding: NOT FOUND (privately held)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -3613,7 +3915,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>RPM / RTM device partner</t>
+          <t>RPM/RTM partner</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
@@ -3633,8 +3935,16 @@
           <t>Independent (private)</t>
         </is>
       </c>
-      <c r="J48" s="3" t="inlineStr"/>
-      <c r="K48" s="3" t="inlineStr"/>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>Tenovi provides 50+ cellular-connected RPM hardware devices with plug-and-play Cellular Gateway. Devices include BP monitors (with wrist BPM option via Jumper Wrist BPM), pulse oximeters, glucose meters, scales, thermometers. Wrist BP monitor is optional arm-cuff alternative, not a smartwatch-style device.</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
       <c r="L48" s="3" t="inlineStr">
         <is>
           <t>https://www.tenovi.com</t>
@@ -3655,7 +3965,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P48" s="3" t="inlineStr"/>
+      <c r="P48" s="3" t="inlineStr">
+        <is>
+          <t>funding: $4.68M raised (3 rounds)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -3673,7 +3987,7 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Smartwatch for medical applications</t>
+          <t>Smartwatch for medical apps</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
@@ -3690,7 +4004,7 @@
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>Shenzhen iWOWN Technology Co., Ltd. (NOT FOUND)</t>
+          <t>Shenzhen iWOWN Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
@@ -3700,8 +4014,7 @@
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND
-N/A</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="L49" s="3" t="inlineStr">
@@ -3716,8 +4029,7 @@
       </c>
       <c r="N49" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND (minimal English-language media presence)
-N/A</t>
+          <t>NOT FOUND (minimal English-language media presence)</t>
         </is>
       </c>
       <c r="O49" s="3" t="inlineStr">
@@ -3747,7 +4059,7 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>eClinical patient monitoring</t>
+          <t>eClinical monitoring</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
@@ -3764,13 +4076,17 @@
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>Independent (N/A)</t>
-        </is>
-      </c>
-      <c r="J50" s="3" t="inlineStr"/>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>eCOA/ePRO platform with smartphone apps, wearable and in-home sensors. Integrates third-party wearables but does not develop proprietary wrist devices.</t>
+        </is>
+      </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>https://getlatka.com/companies/datacubed.com</t>
         </is>
       </c>
       <c r="L50" s="3" t="inlineStr">
@@ -3788,8 +4104,16 @@
           <t>Datacubed Health Sharpens Focus on eCOA and ePRO With New CEO — Yahoo Finance / BioSpace, 2025 — https://finance.yahoo.com/news/datacubed-health-sharpens-focus-ecoa-120000767.html</t>
         </is>
       </c>
-      <c r="O50" s="3" t="inlineStr"/>
-      <c r="P50" s="3" t="inlineStr"/>
+      <c r="O50" s="3" t="inlineStr">
+        <is>
+          <t>Seed-list exception</t>
+        </is>
+      </c>
+      <c r="P50" s="3" t="inlineStr">
+        <is>
+          <t>wrist_device_core=False</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -3807,7 +4131,7 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Remote monitoring + devices</t>
+          <t>Remote monitoring</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
@@ -3824,13 +4148,17 @@
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>Independent (private)</t>
-        </is>
-      </c>
-      <c r="J51" s="3" t="inlineStr"/>
+          <t>Independent (private) (~$500K TTM revenue)</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>HealthArc provides cellular medical devices for RPM including BP monitors, glucose meters, pulse oximeters, and scales. No wrist-worn device identified.</t>
+        </is>
+      </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t>~$500K TTM revenue
 https://gust.com/companies/healtharc</t>
         </is>
       </c>
@@ -3854,7 +4182,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P51" s="3" t="inlineStr"/>
+      <c r="P51" s="3" t="inlineStr">
+        <is>
+          <t>funding: NOT FOUND</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -3872,7 +4204,7 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Corporate wellness + wearables</t>
+          <t>Corporate wellness</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
@@ -3889,13 +4221,17 @@
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>Independent (bootstrapped)</t>
-        </is>
-      </c>
-      <c r="J52" s="3" t="inlineStr"/>
+          <t>Independent (bootstrapped) ($2.5M ARR (2025))</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>IncentFit provides corporate wellness software for challenges, reimbursements, and fitness rewards. Platform integrates with fitness apps and wearables but does not deploy its own wrist-worn devices.</t>
+        </is>
+      </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t>$2.5M ARR (2025)
 https://getlatka.com/companies/incentfit.com</t>
         </is>
       </c>
@@ -3919,7 +4255,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P52" s="3" t="inlineStr"/>
+      <c r="P52" s="3" t="inlineStr">
+        <is>
+          <t>funding: $20K seed (bootstrapped)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -3954,7 +4294,7 @@
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>VOSPV LLC (NOT FOUND)</t>
+          <t>VOSPV LLC</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
@@ -3964,8 +4304,7 @@
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND
-N/A</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="L53" s="3" t="inlineStr">
@@ -3980,8 +4319,7 @@
       </c>
       <c r="N53" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND (minimal media presence)
-N/A</t>
+          <t>NOT FOUND (minimal media presence)</t>
         </is>
       </c>
       <c r="O53" s="3" t="inlineStr">
@@ -4011,7 +4349,7 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Device-data layer + wearables</t>
+          <t>Device-data layer</t>
         </is>
       </c>
       <c r="E54" s="2" t="n">
@@ -4028,11 +4366,19 @@
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>Independent (LLC formed June 2026)</t>
-        </is>
-      </c>
-      <c r="J54" s="3" t="inlineStr"/>
-      <c r="K54" s="3" t="inlineStr"/>
+          <t>Independent (LLC formed June 2026) (NOT FOUND (newly incorporated))</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>OVRVEW is a device-data layer for RPM — they collect and normalize readings from approved connected devices. They offer white-label FDA-cleared cellular devices but their model is data infrastructure, not device deployment. No evidence of wrist-worn device deployment.</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>NOT FOUND (newly incorporated)</t>
+        </is>
+      </c>
       <c r="L54" s="3" t="inlineStr">
         <is>
           <t>https://ovrvew.com</t>
@@ -4053,7 +4399,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P54" s="3" t="inlineStr"/>
+      <c r="P54" s="3" t="inlineStr">
+        <is>
+          <t>funding: NOT FOUND (newly formed LLC)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -4071,7 +4421,7 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Employee challenge platform</t>
+          <t>Employee challenges</t>
         </is>
       </c>
       <c r="E55" s="2" t="n">
@@ -4091,8 +4441,16 @@
           <t>Independent (private, founded 2013)</t>
         </is>
       </c>
-      <c r="J55" s="3" t="inlineStr"/>
-      <c r="K55" s="3" t="inlineStr"/>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>ReachingApp syncs with Apple Health, Fitbit, Garmin, Google Fit, and Apple Watch for step tracking in wellness challenges. Does not deploy own wrist-worn devices.</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
       <c r="L55" s="3" t="inlineStr">
         <is>
           <t>https://www.reachingapp.com</t>
@@ -4113,7 +4471,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P55" s="3" t="inlineStr"/>
+      <c r="P55" s="3" t="inlineStr">
+        <is>
+          <t>funding: NOT FOUND</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -4131,7 +4493,7 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Step-challenge platform</t>
+          <t>Step-challenge</t>
         </is>
       </c>
       <c r="E56" s="2" t="n">
@@ -4151,8 +4513,16 @@
           <t>Independent (private)</t>
         </is>
       </c>
-      <c r="J56" s="3" t="inlineStr"/>
-      <c r="K56" s="3" t="inlineStr"/>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>STEPPI integrates with compatible Garmin wearable devices for corporate wellness challenges and step tracking. Does not deploy its own wrist-worn devices; relies on consumer wearables.</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
       <c r="L56" s="3" t="inlineStr">
         <is>
           <t>https://www.steppi.com</t>
@@ -4173,7 +4543,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P56" s="3" t="inlineStr"/>
+      <c r="P56" s="3" t="inlineStr">
+        <is>
+          <t>funding: $1.8M raised (2021 corporate round)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -4191,7 +4565,7 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Employee movement platform</t>
+          <t>Employee movement</t>
         </is>
       </c>
       <c r="E57" s="2" t="n">
@@ -4211,8 +4585,16 @@
           <t>Independent (private)</t>
         </is>
       </c>
-      <c r="J57" s="3" t="inlineStr"/>
-      <c r="K57" s="3" t="inlineStr"/>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>Teamupp is a corporate wellness and team building platform for challenges and activities. No evidence of deploying wrist-worn devices. Focus is on challenge management and team cohesion.</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
       <c r="L57" s="3" t="inlineStr">
         <is>
           <t>https://teamupp.io</t>
@@ -4233,7 +4615,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P57" s="3" t="inlineStr"/>
+      <c r="P57" s="3" t="inlineStr">
+        <is>
+          <t>funding: NOT FOUND</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -4251,7 +4637,7 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Corporate wellness + wearables</t>
+          <t>Corporate wellness</t>
         </is>
       </c>
       <c r="E58" s="2" t="n">
@@ -4268,13 +4654,17 @@
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>Independent (bootstrapped)</t>
-        </is>
-      </c>
-      <c r="J58" s="3" t="inlineStr"/>
+          <t>Independent (bootstrapped) ($4.3M (bootstrapped))</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>Woliba is a corporate wellness and engagement platform that syncs with wearables (Fitbit, Apple Watch, Garmin) for step tracking and wellness challenges. Does not deploy or provide its own wrist-worn devices.</t>
+        </is>
+      </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t>$4.3M (bootstrapped)
 https://getlatka.com/companies/woliba.io</t>
         </is>
       </c>
@@ -4298,7 +4688,11 @@
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="P58" s="3" t="inlineStr"/>
+      <c r="P58" s="3" t="inlineStr">
+        <is>
+          <t>funding: $0 (bootstrapped, no outside funding)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4382,7 +4776,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Not critical — wrist device peripheral or absent</t>
+          <t>Not critical — wrist device peripheral/absent</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -4392,7 +4786,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Minimal / no recent coverage</t>
+          <t>Minimal coverage</t>
         </is>
       </c>
     </row>
@@ -4404,7 +4798,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Somewhat — wrist important but not sole device</t>
+          <t>Somewhat — wrist important but not sole</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -4426,7 +4820,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Critical — wrist device is core product, wrong fit = clinical data failure at scale</t>
+          <t>Critical — wrist core, wrong fit = clinical failure at scale</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -4666,7 +5060,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Top 10 — Highest Priority</t>
+          <t>Top 10</t>
         </is>
       </c>
     </row>
@@ -4723,7 +5117,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Insurance wellness / rewards</t>
+          <t>Insurance wellness rewards</t>
         </is>
       </c>
       <c r="D25" s="2" t="n">
@@ -4787,7 +5181,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Wearable DHT for clinical trials</t>
+          <t>Wearable DHT clinical trials</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
@@ -4819,7 +5213,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>RPM + clinical trials (wrist)</t>
+          <t>RPM + trials (wrist)</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
@@ -4836,7 +5230,7 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>Independent (life sciences division acquired by ActiGraph Jan 2025) (N/A)</t>
+          <t>Independent (life sciences division acquired by ActiGraph Jan 2025)</t>
         </is>
       </c>
     </row>
@@ -4851,7 +5245,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Endpoint data + wearable sensors</t>
+          <t>Endpoint data + wearables</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
@@ -4883,7 +5277,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Insurer rewards ecosystem</t>
+          <t>Insurer rewards</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
@@ -4915,7 +5309,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Unified trial solution + RPM</t>
+          <t>Unified trial + RPM</t>
         </is>
       </c>
       <c r="D31" s="2" t="n">
@@ -4964,7 +5358,7 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>None (public: NASDAQ MASI) (N/A)</t>
+          <t>None (public: NASDAQ MASI)</t>
         </is>
       </c>
     </row>
@@ -5011,7 +5405,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Employer wellbeing platform</t>
+          <t>Employer wellbeing</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
@@ -5052,7 +5446,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>No companies excluded — all 57 were researched and scored.</t>
+          <t>No excluded companies — all 57 researched and scored.</t>
         </is>
       </c>
     </row>
@@ -5067,12 +5461,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
@@ -5080,7 +5474,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Needs Verification / Verification Failed</t>
+          <t>Needs Verification / Data Gaps</t>
         </is>
       </c>
     </row>
@@ -5102,7 +5496,7 @@
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>D2C/B2B?</t>
+          <t>E-com</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -5114,17 +5508,17 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Betterfly</t>
+          <t>Evinova</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Insurtech / wellbeing app</t>
+          <t>Unified trial + RPM</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Wrist device not confirmed</t>
+          <t>No proprietary wrist device</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -5133,23 +5527,23 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Luscii</t>
+          <t>Betterfly</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Remote monitoring platform</t>
+          <t>Insurtech wellbeing</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Wrist device not confirmed</t>
+          <t>No proprietary wrist device</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -5158,23 +5552,23 @@
         </is>
       </c>
       <c r="E5" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>CardiacSense</t>
+          <t>Doccla</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Medical watch + doctor portal</t>
+          <t>Virtual wards</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Needs further verification</t>
+          <t>Revenue data not found</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -5183,23 +5577,23 @@
         </is>
       </c>
       <c r="E6" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>ClearPath RPM</t>
+          <t>ICON plc</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>RPM watch + clinician dashboard</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Needs further verification</t>
+          <t>No proprietary wrist device</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -5208,23 +5602,23 @@
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>CoachCare</t>
+          <t>IQVIA</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>RPM / RTM platform</t>
+          <t>CRO / trial-tech</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Wrist device not confirmed</t>
+          <t>No proprietary wrist device</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -5233,23 +5627,23 @@
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Health Recovery Solutions (HRS)</t>
+          <t>Medable</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Decentralized trials</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Revenue data not found; Wrist device not confirmed</t>
+          <t>No proprietary wrist device</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -5258,23 +5652,23 @@
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>100Plus</t>
+          <t>Medidata</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Remote care + shipped devices</t>
+          <t>Sensor platform trials</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Wrist device not confirmed</t>
+          <t>No proprietary wrist device</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -5283,23 +5677,23 @@
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>AMC Health</t>
+          <t>Parexel</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Home monitoring kits</t>
+          <t>CRO DCT wearables</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Revenue data not found; Wrist device not confirmed</t>
+          <t>No proprietary wrist device</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -5308,23 +5702,23 @@
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>HUSK Wellness</t>
+          <t>Science 37</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Workplace challenges</t>
+          <t>Direct-to-patient trials</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Wrist device not confirmed</t>
+          <t>No proprietary wrist device</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -5333,23 +5727,23 @@
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>HeiaHeia</t>
+          <t>Castor</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Employee wellbeing platform</t>
+          <t>Decentralized/hybrid trials</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Wrist device not confirmed</t>
+          <t>No proprietary wrist device</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -5358,23 +5752,23 @@
         </is>
       </c>
       <c r="E13" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Prevounce Health</t>
+          <t>Koneksa Health</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Remote care + cellular devices</t>
+          <t>Digital biomarker wearable</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Wrist device not confirmed</t>
+          <t>No proprietary wrist device</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -5383,23 +5777,23 @@
         </is>
       </c>
       <c r="E14" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Smart Meter</t>
+          <t>Luscii</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Cellular RPM device network</t>
+          <t>Remote monitoring</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Revenue data not found; Wrist device not confirmed</t>
+          <t>No proprietary wrist device</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -5408,23 +5802,23 @@
         </is>
       </c>
       <c r="E15" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Tenovi</t>
+          <t>dacadoo</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>RPM / RTM device partner</t>
+          <t>Health engagement platform</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Revenue data not found; Wrist device not confirmed</t>
+          <t>No proprietary wrist device</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -5433,48 +5827,48 @@
         </is>
       </c>
       <c r="E16" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>iWOWN</t>
+          <t>yulife</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Smartwatch for medical applications</t>
+          <t>Group insurance wellbeing</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Needs further verification</t>
+          <t>No proprietary wrist device</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>B2B+B2C</t>
+          <t>B2B</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>HealthArc</t>
+          <t>CardiacSense</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Remote monitoring + devices</t>
+          <t>Medical watch + doctor portal</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Wrist device not confirmed</t>
+          <t>Revenue data not found</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -5483,23 +5877,23 @@
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>IncentFit</t>
+          <t>ClearPath RPM</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Corporate wellness + wearables</t>
+          <t>RPM watch + clinician dashboard</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Wrist device not confirmed</t>
+          <t>Revenue data not found</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -5508,23 +5902,23 @@
         </is>
       </c>
       <c r="E19" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>OVRVEW</t>
+          <t>CoachCare</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Device-data layer + wearables</t>
+          <t>RPM/RTM platform</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Revenue data not found; Wrist device not confirmed</t>
+          <t>No proprietary wrist device</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -5533,23 +5927,23 @@
         </is>
       </c>
       <c r="E20" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>ReachingApp</t>
+          <t>Corsano Health</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Employee challenge platform</t>
+          <t>Wrist bracelet for RPM + research</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Revenue data not found; Wrist device not confirmed</t>
+          <t>Revenue data not found</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -5558,23 +5952,23 @@
         </is>
       </c>
       <c r="E21" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>STEPPI</t>
+          <t>Curebase</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Step-challenge platform</t>
+          <t>Remote trial platform</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Revenue data not found; Wrist device not confirmed</t>
+          <t>No proprietary wrist device</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -5583,23 +5977,23 @@
         </is>
       </c>
       <c r="E22" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Teamupp</t>
+          <t>Health Recovery Solutions (HRS)</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Employee movement platform</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Revenue data not found; Wrist device not confirmed</t>
+          <t>Revenue data not found; No proprietary wrist device</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -5608,31 +6002,531 @@
         </is>
       </c>
       <c r="E23" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
+          <t>ObvioHealth</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Digital DCT platform</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>THREAD</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>DHT decentralized trials</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Validic</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Wearable data API + RPM</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>100Plus</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Remote care+devices</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>AMC Health</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Home monitoring kits</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Revenue data not found; No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>HUSK Wellness</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Workplace challenges</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>HeiaHeia</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Employee wellbeing</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>My Medic Watch</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Provider monitoring via smartwatches</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Revenue data not found</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Prevounce Health</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Remote care+cellular</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Smart Meter</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Cellular RPM network</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Tenovi</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>RPM/RTM partner</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Revenue data not found; No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>iWOWN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Smartwatch for medical apps</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Revenue data not found</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>B2B+B2C</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Datacubed Health</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>eClinical monitoring</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>HealthArc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Remote monitoring</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>IncentFit</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Corporate wellness</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>MedRPM</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>RPM platform with wearables</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Revenue data not found; No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>OVRVEW</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Device-data layer</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>ReachingApp</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Employee challenges</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Revenue data not found; No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>STEPPI</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Step-challenge</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Revenue data not found; No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Teamupp</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Employee movement</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Revenue data not found; No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
           <t>Woliba</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Corporate wellness + wearables</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Wrist device not confirmed</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>B2B</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="n">
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Corporate wellness</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>No proprietary wrist device</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>